<commit_message>
added new data in AVP and Tribunales
</commit_message>
<xml_diff>
--- a/data/Administracion_de_viviendas_publicas/datos_vivienda.xlsx
+++ b/data/Administracion_de_viviendas_publicas/datos_vivienda.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Administracion_de_viviendas_publicas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29B47C1E-6D21-48AF-A626-F80B89258D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59D27232-8002-46D8-BDBF-16430A4EB2F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" tabRatio="847" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="municipios_soli" sheetId="1" r:id="rId1"/>
@@ -903,14 +903,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:K79"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>81</v>
       </c>
@@ -941,8 +941,11 @@
       <c r="J1" s="1">
         <v>2024</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K1" s="1">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -973,8 +976,11 @@
       <c r="J2">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1005,8 +1011,11 @@
       <c r="J3">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1037,8 +1046,11 @@
       <c r="J4">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1069,8 +1081,11 @@
       <c r="J5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1101,8 +1116,11 @@
       <c r="J6">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1133,8 +1151,11 @@
       <c r="J7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1165,8 +1186,11 @@
       <c r="J8">
         <v>9</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1197,8 +1221,11 @@
       <c r="J9">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1229,8 +1256,11 @@
       <c r="J10">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1261,8 +1291,11 @@
       <c r="J11">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>64</v>
       </c>
@@ -1293,8 +1326,11 @@
       <c r="J12">
         <v>34</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K12">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1325,8 +1361,11 @@
       <c r="J13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1357,8 +1396,11 @@
       <c r="J14">
         <v>16</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K14">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1389,8 +1431,11 @@
       <c r="J15">
         <v>3</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -1421,8 +1466,11 @@
       <c r="J16">
         <v>10</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -1453,8 +1501,11 @@
       <c r="J17">
         <v>32</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K17">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>66</v>
       </c>
@@ -1485,8 +1536,11 @@
       <c r="J18">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -1517,8 +1571,11 @@
       <c r="J19">
         <v>7</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -1549,8 +1606,11 @@
       <c r="J20">
         <v>2</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -1581,8 +1641,11 @@
       <c r="J21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>18</v>
       </c>
@@ -1613,8 +1676,11 @@
       <c r="J22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K22">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>19</v>
       </c>
@@ -1645,8 +1711,11 @@
       <c r="J23">
         <v>4</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>67</v>
       </c>
@@ -1677,8 +1746,11 @@
       <c r="J24">
         <v>9</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K24">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>20</v>
       </c>
@@ -1709,8 +1781,11 @@
       <c r="J25">
         <v>2</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>79</v>
       </c>
@@ -1741,8 +1816,11 @@
       <c r="J26">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -1773,8 +1851,11 @@
       <c r="J27">
         <v>5</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K27">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -1805,8 +1886,11 @@
       <c r="J28">
         <v>9</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K28">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -1837,8 +1921,11 @@
       <c r="J29">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>68</v>
       </c>
@@ -1869,8 +1956,11 @@
       <c r="J30">
         <v>5</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>24</v>
       </c>
@@ -1901,8 +1991,11 @@
       <c r="J31">
         <v>18</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K31">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>25</v>
       </c>
@@ -1933,8 +2026,11 @@
       <c r="J32">
         <v>5</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>26</v>
       </c>
@@ -1965,8 +2061,11 @@
       <c r="J33">
         <v>10</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K33">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>27</v>
       </c>
@@ -1997,8 +2096,11 @@
       <c r="J34">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>28</v>
       </c>
@@ -2029,8 +2131,11 @@
       <c r="J35">
         <v>2</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>29</v>
       </c>
@@ -2061,8 +2166,11 @@
       <c r="J36">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>30</v>
       </c>
@@ -2093,8 +2201,11 @@
       <c r="J37">
         <v>9</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K37">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>31</v>
       </c>
@@ -2125,8 +2236,11 @@
       <c r="J38">
         <v>2</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>32</v>
       </c>
@@ -2157,8 +2271,11 @@
       <c r="J39">
         <v>3</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>69</v>
       </c>
@@ -2189,8 +2306,11 @@
       <c r="J40">
         <v>1</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>33</v>
       </c>
@@ -2221,8 +2341,11 @@
       <c r="J41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K41">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>34</v>
       </c>
@@ -2253,8 +2376,11 @@
       <c r="J42">
         <v>1</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>35</v>
       </c>
@@ -2285,8 +2411,11 @@
       <c r="J43">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K43">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>36</v>
       </c>
@@ -2317,8 +2446,11 @@
       <c r="J44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>37</v>
       </c>
@@ -2349,8 +2481,11 @@
       <c r="J45">
         <v>4</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>70</v>
       </c>
@@ -2381,8 +2516,11 @@
       <c r="J46">
         <v>2</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>38</v>
       </c>
@@ -2413,8 +2551,11 @@
       <c r="J47">
         <v>3</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K47">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>71</v>
       </c>
@@ -2445,8 +2586,11 @@
       <c r="J48">
         <v>5</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>39</v>
       </c>
@@ -2477,8 +2621,11 @@
       <c r="J49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>40</v>
       </c>
@@ -2509,8 +2656,11 @@
       <c r="J50">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>78</v>
       </c>
@@ -2541,8 +2691,11 @@
       <c r="J51">
         <v>11</v>
       </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K51">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>41</v>
       </c>
@@ -2573,8 +2726,11 @@
       <c r="J52">
         <v>1</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K52">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>42</v>
       </c>
@@ -2605,8 +2761,11 @@
       <c r="J53">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>43</v>
       </c>
@@ -2637,8 +2796,11 @@
       <c r="J54">
         <v>2</v>
       </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K54">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>44</v>
       </c>
@@ -2669,8 +2831,11 @@
       <c r="J55">
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>45</v>
       </c>
@@ -2701,8 +2866,11 @@
       <c r="J56">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K56">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>46</v>
       </c>
@@ -2733,8 +2901,11 @@
       <c r="J57">
         <v>4</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>72</v>
       </c>
@@ -2765,8 +2936,11 @@
       <c r="J58">
         <v>1</v>
       </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>47</v>
       </c>
@@ -2797,8 +2971,11 @@
       <c r="J59">
         <v>36</v>
       </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K59">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>48</v>
       </c>
@@ -2829,8 +3006,11 @@
       <c r="J60">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>73</v>
       </c>
@@ -2861,8 +3041,11 @@
       <c r="J61">
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>74</v>
       </c>
@@ -2893,8 +3076,11 @@
       <c r="J62">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K62">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>49</v>
       </c>
@@ -2925,8 +3111,11 @@
       <c r="J63">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>50</v>
       </c>
@@ -2957,8 +3146,11 @@
       <c r="J64">
         <v>6</v>
       </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K64">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>75</v>
       </c>
@@ -2989,8 +3181,11 @@
       <c r="J65">
         <v>1</v>
       </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K65">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>51</v>
       </c>
@@ -3021,8 +3216,11 @@
       <c r="J66">
         <v>69</v>
       </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K66">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>52</v>
       </c>
@@ -3053,8 +3251,11 @@
       <c r="J67">
         <v>0</v>
       </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K67">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>76</v>
       </c>
@@ -3085,8 +3286,11 @@
       <c r="J68">
         <v>3</v>
       </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K68">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>53</v>
       </c>
@@ -3117,8 +3321,11 @@
       <c r="J69">
         <v>0</v>
       </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K69">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>54</v>
       </c>
@@ -3149,8 +3356,11 @@
       <c r="J70">
         <v>3</v>
       </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K70">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>55</v>
       </c>
@@ -3181,8 +3391,11 @@
       <c r="J71">
         <v>4</v>
       </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>56</v>
       </c>
@@ -3213,8 +3426,11 @@
       <c r="J72">
         <v>9</v>
       </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K72">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>57</v>
       </c>
@@ -3245,8 +3461,11 @@
       <c r="J73">
         <v>2</v>
       </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K73">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>58</v>
       </c>
@@ -3277,8 +3496,11 @@
       <c r="J74">
         <v>5</v>
       </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K74">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>59</v>
       </c>
@@ -3309,8 +3531,11 @@
       <c r="J75">
         <v>2</v>
       </c>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>60</v>
       </c>
@@ -3341,8 +3566,11 @@
       <c r="J76">
         <v>0</v>
       </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K76">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>61</v>
       </c>
@@ -3373,8 +3601,11 @@
       <c r="J77">
         <v>4</v>
       </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K77">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>62</v>
       </c>
@@ -3405,8 +3636,11 @@
       <c r="J78">
         <v>1</v>
       </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K78">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>63</v>
       </c>
@@ -3436,6 +3670,9 @@
       </c>
       <c r="J79">
         <v>3</v>
+      </c>
+      <c r="K79">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -3446,14 +3683,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:K79"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>81</v>
       </c>
@@ -3484,8 +3721,11 @@
       <c r="J1" s="1">
         <v>2024</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K1" s="1">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3516,8 +3756,11 @@
       <c r="J2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -3548,8 +3791,11 @@
       <c r="J3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -3580,8 +3826,11 @@
       <c r="J4">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -3612,8 +3861,11 @@
       <c r="J5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -3644,8 +3896,11 @@
       <c r="J6">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -3676,8 +3931,11 @@
       <c r="J7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -3708,8 +3966,11 @@
       <c r="J8">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -3740,8 +4001,11 @@
       <c r="J9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -3772,8 +4036,11 @@
       <c r="J10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3804,8 +4071,11 @@
       <c r="J11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>64</v>
       </c>
@@ -3836,8 +4106,11 @@
       <c r="J12">
         <v>18</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K12">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -3868,8 +4141,11 @@
       <c r="J13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -3900,8 +4176,11 @@
       <c r="J14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K14">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -3932,8 +4211,11 @@
       <c r="J15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -3964,8 +4246,11 @@
       <c r="J16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -3996,8 +4281,11 @@
       <c r="J17">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K17">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>66</v>
       </c>
@@ -4028,8 +4316,11 @@
       <c r="J18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -4060,8 +4351,11 @@
       <c r="J19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -4092,8 +4386,11 @@
       <c r="J20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -4124,8 +4421,11 @@
       <c r="J21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>18</v>
       </c>
@@ -4156,8 +4456,11 @@
       <c r="J22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K22">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>19</v>
       </c>
@@ -4188,8 +4491,11 @@
       <c r="J23">
         <v>2</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>67</v>
       </c>
@@ -4220,8 +4526,11 @@
       <c r="J24">
         <v>2</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>20</v>
       </c>
@@ -4252,8 +4561,11 @@
       <c r="J25">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>79</v>
       </c>
@@ -4284,8 +4596,11 @@
       <c r="J26">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -4316,8 +4631,11 @@
       <c r="J27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -4348,8 +4666,11 @@
       <c r="J28">
         <v>2</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -4380,8 +4701,11 @@
       <c r="J29">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>68</v>
       </c>
@@ -4412,8 +4736,11 @@
       <c r="J30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>24</v>
       </c>
@@ -4444,8 +4771,11 @@
       <c r="J31">
         <v>10</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K31">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>25</v>
       </c>
@@ -4476,8 +4806,11 @@
       <c r="J32">
         <v>3</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>26</v>
       </c>
@@ -4508,8 +4841,11 @@
       <c r="J33">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>27</v>
       </c>
@@ -4540,8 +4876,11 @@
       <c r="J34">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>28</v>
       </c>
@@ -4572,8 +4911,11 @@
       <c r="J35">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>29</v>
       </c>
@@ -4604,8 +4946,11 @@
       <c r="J36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>30</v>
       </c>
@@ -4636,8 +4981,11 @@
       <c r="J37">
         <v>6</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K37">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>31</v>
       </c>
@@ -4668,8 +5016,11 @@
       <c r="J38">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>32</v>
       </c>
@@ -4700,8 +5051,11 @@
       <c r="J39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>69</v>
       </c>
@@ -4732,8 +5086,11 @@
       <c r="J40">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>33</v>
       </c>
@@ -4764,8 +5121,11 @@
       <c r="J41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K41">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>34</v>
       </c>
@@ -4796,8 +5156,11 @@
       <c r="J42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>35</v>
       </c>
@@ -4828,8 +5191,11 @@
       <c r="J43">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>36</v>
       </c>
@@ -4860,8 +5226,11 @@
       <c r="J44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>37</v>
       </c>
@@ -4892,8 +5261,11 @@
       <c r="J45">
         <v>2</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>70</v>
       </c>
@@ -4924,8 +5296,11 @@
       <c r="J46">
         <v>1</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>38</v>
       </c>
@@ -4956,8 +5331,11 @@
       <c r="J47">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K47">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>71</v>
       </c>
@@ -4988,8 +5366,11 @@
       <c r="J48">
         <v>4</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K48">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>39</v>
       </c>
@@ -5020,8 +5401,11 @@
       <c r="J49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>40</v>
       </c>
@@ -5052,8 +5436,11 @@
       <c r="J50">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>78</v>
       </c>
@@ -5084,8 +5471,11 @@
       <c r="J51">
         <v>9</v>
       </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K51">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>41</v>
       </c>
@@ -5116,8 +5506,11 @@
       <c r="J52">
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>42</v>
       </c>
@@ -5148,8 +5541,11 @@
       <c r="J53">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>43</v>
       </c>
@@ -5180,8 +5576,11 @@
       <c r="J54">
         <v>1</v>
       </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K54">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>44</v>
       </c>
@@ -5212,8 +5611,11 @@
       <c r="J55">
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>45</v>
       </c>
@@ -5244,8 +5646,11 @@
       <c r="J56">
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>46</v>
       </c>
@@ -5276,8 +5681,11 @@
       <c r="J57">
         <v>1</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>72</v>
       </c>
@@ -5308,8 +5716,11 @@
       <c r="J58">
         <v>0</v>
       </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>47</v>
       </c>
@@ -5340,8 +5751,11 @@
       <c r="J59">
         <v>26</v>
       </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K59">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>48</v>
       </c>
@@ -5372,8 +5786,11 @@
       <c r="J60">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>73</v>
       </c>
@@ -5404,8 +5821,11 @@
       <c r="J61">
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>74</v>
       </c>
@@ -5436,8 +5856,11 @@
       <c r="J62">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>49</v>
       </c>
@@ -5468,8 +5891,11 @@
       <c r="J63">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>50</v>
       </c>
@@ -5500,8 +5926,11 @@
       <c r="J64">
         <v>2</v>
       </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>75</v>
       </c>
@@ -5532,8 +5961,11 @@
       <c r="J65">
         <v>1</v>
       </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K65">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>51</v>
       </c>
@@ -5564,8 +5996,11 @@
       <c r="J66">
         <v>38</v>
       </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K66">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>52</v>
       </c>
@@ -5596,8 +6031,11 @@
       <c r="J67">
         <v>0</v>
       </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>76</v>
       </c>
@@ -5628,8 +6066,11 @@
       <c r="J68">
         <v>3</v>
       </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K68">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>53</v>
       </c>
@@ -5660,8 +6101,11 @@
       <c r="J69">
         <v>0</v>
       </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K69">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>54</v>
       </c>
@@ -5692,8 +6136,11 @@
       <c r="J70">
         <v>0</v>
       </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>55</v>
       </c>
@@ -5724,8 +6171,11 @@
       <c r="J71">
         <v>3</v>
       </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>56</v>
       </c>
@@ -5756,8 +6206,11 @@
       <c r="J72">
         <v>2</v>
       </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K72">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>57</v>
       </c>
@@ -5788,8 +6241,11 @@
       <c r="J73">
         <v>1</v>
       </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>58</v>
       </c>
@@ -5820,8 +6276,11 @@
       <c r="J74">
         <v>2</v>
       </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K74">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>59</v>
       </c>
@@ -5852,8 +6311,11 @@
       <c r="J75">
         <v>0</v>
       </c>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>60</v>
       </c>
@@ -5884,8 +6346,11 @@
       <c r="J76">
         <v>0</v>
       </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K76">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>61</v>
       </c>
@@ -5916,8 +6381,11 @@
       <c r="J77">
         <v>3</v>
       </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>62</v>
       </c>
@@ -5948,8 +6416,11 @@
       <c r="J78">
         <v>1</v>
       </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K78">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>63</v>
       </c>
@@ -5979,6 +6450,9 @@
       </c>
       <c r="J79">
         <v>3</v>
+      </c>
+      <c r="K79">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -5988,13 +6462,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
@@ -6022,8 +6496,11 @@
       <c r="I1" s="1">
         <v>2024</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J1" s="1">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -6051,8 +6528,11 @@
       <c r="I2">
         <v>34</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6080,8 +6560,11 @@
       <c r="I3">
         <v>38</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -6107,10 +6590,13 @@
         <v>58</v>
       </c>
       <c r="I4">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+      <c r="J4">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -6138,8 +6624,11 @@
       <c r="I5">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J5">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -6167,8 +6656,11 @@
       <c r="I6">
         <v>65</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J6">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -6196,8 +6688,11 @@
       <c r="I7">
         <v>39</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J7">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -6225,8 +6720,11 @@
       <c r="I8">
         <v>19</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>78</v>
       </c>
@@ -6254,8 +6752,11 @@
       <c r="I9">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J9">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -6281,10 +6782,13 @@
         <v>33</v>
       </c>
       <c r="I10">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+      <c r="J10">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>51</v>
       </c>
@@ -6311,6 +6815,9 @@
       </c>
       <c r="I11">
         <v>69</v>
+      </c>
+      <c r="J11">
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -6323,13 +6830,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
@@ -6357,8 +6864,11 @@
       <c r="I1" s="1">
         <v>2024</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J1" s="1">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -6386,8 +6896,11 @@
       <c r="I2">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6415,8 +6928,11 @@
       <c r="I3">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -6444,8 +6960,11 @@
       <c r="I4">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J4">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -6473,8 +6992,11 @@
       <c r="I5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -6502,8 +7024,11 @@
       <c r="I6">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -6529,10 +7054,13 @@
         <v>4</v>
       </c>
       <c r="I7">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="J7">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -6560,8 +7088,11 @@
       <c r="I8">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>78</v>
       </c>
@@ -6589,8 +7120,11 @@
       <c r="I9">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J9">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -6616,10 +7150,13 @@
         <v>21</v>
       </c>
       <c r="I10">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+      <c r="J10">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>51</v>
       </c>
@@ -6646,6 +7183,9 @@
       </c>
       <c r="I11">
         <v>38</v>
+      </c>
+      <c r="J11">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>